<commit_message>
fix(MM nonlinearities): Km_P should have C1 units, P_min should have P units
</commit_message>
<xml_diff>
--- a/pkpdapp/pkpdapp/migrations/models/ParametersValue_Species.xlsx
+++ b/pkpdapp/pkpdapp/migrations/models/ParametersValue_Species.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrobins/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CD79781-C6AF-F84D-BF76-769FDE5D67D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5289CC86-B9E5-964C-86A6-4992113DF6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="1200" windowWidth="29020" windowHeight="18880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4360" yWindow="1200" windowWidth="29020" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1cmpt_PK_Model" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="51">
   <si>
     <t>SM_Mouse</t>
   </si>
@@ -182,6 +182,18 @@
   </si>
   <si>
     <t>µg/h/kg</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>µg/mL</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
   </si>
 </sst>
 </file>
@@ -551,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
@@ -1133,6 +1145,43 @@
         <v>29</v>
       </c>
     </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="5"/>
+      <c r="I12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J12" s="5"/>
+      <c r="K12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L12" s="5"/>
+      <c r="M12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N12" s="5"/>
+      <c r="O12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1141,7 +1190,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
@@ -1867,6 +1916,80 @@
         <v>29</v>
       </c>
     </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H14" s="5"/>
+      <c r="I14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J14" s="5"/>
+      <c r="K14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L14" s="5"/>
+      <c r="M14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N14" s="5"/>
+      <c r="O14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H15" s="5"/>
+      <c r="I15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="5"/>
+      <c r="K15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L15" s="5"/>
+      <c r="M15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N15" s="5"/>
+      <c r="O15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1875,7 +1998,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
@@ -2735,6 +2858,117 @@
       </c>
       <c r="Q15" s="3" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J16" s="5"/>
+      <c r="K16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L16" s="5"/>
+      <c r="M16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N16" s="5"/>
+      <c r="O16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" s="5"/>
+      <c r="I17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J17" s="5"/>
+      <c r="K17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L17" s="5"/>
+      <c r="M17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N17" s="5"/>
+      <c r="O17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J18" s="5"/>
+      <c r="K18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L18" s="5"/>
+      <c r="M18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N18" s="5"/>
+      <c r="O18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(MM Nonlin): Km should have units of secondary var, _min should have units of primary var (#1117)
* fix(MM nonlinearities): Km_P should have C1 units, P_min should have P units

* fix: remove prints

* fix: test

* increase test timeout
</commit_message>
<xml_diff>
--- a/pkpdapp/pkpdapp/migrations/models/ParametersValue_Species.xlsx
+++ b/pkpdapp/pkpdapp/migrations/models/ParametersValue_Species.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrobins/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CD79781-C6AF-F84D-BF76-769FDE5D67D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5289CC86-B9E5-964C-86A6-4992113DF6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="1200" windowWidth="29020" windowHeight="18880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4360" yWindow="1200" windowWidth="29020" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1cmpt_PK_Model" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="51">
   <si>
     <t>SM_Mouse</t>
   </si>
@@ -182,6 +182,18 @@
   </si>
   <si>
     <t>µg/h/kg</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>µg/mL</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
   </si>
 </sst>
 </file>
@@ -551,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
@@ -1133,6 +1145,43 @@
         <v>29</v>
       </c>
     </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="5"/>
+      <c r="I12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J12" s="5"/>
+      <c r="K12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L12" s="5"/>
+      <c r="M12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N12" s="5"/>
+      <c r="O12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1141,7 +1190,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
@@ -1867,6 +1916,80 @@
         <v>29</v>
       </c>
     </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H14" s="5"/>
+      <c r="I14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J14" s="5"/>
+      <c r="K14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L14" s="5"/>
+      <c r="M14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N14" s="5"/>
+      <c r="O14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H15" s="5"/>
+      <c r="I15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="5"/>
+      <c r="K15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L15" s="5"/>
+      <c r="M15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N15" s="5"/>
+      <c r="O15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1875,7 +1998,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
@@ -2735,6 +2858,117 @@
       </c>
       <c r="Q15" s="3" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J16" s="5"/>
+      <c r="K16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L16" s="5"/>
+      <c r="M16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N16" s="5"/>
+      <c r="O16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" s="5"/>
+      <c r="I17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J17" s="5"/>
+      <c r="K17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L17" s="5"/>
+      <c r="M17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N17" s="5"/>
+      <c r="O17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J18" s="5"/>
+      <c r="K18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L18" s="5"/>
+      <c r="M18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N18" s="5"/>
+      <c r="O18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>